<commit_message>
sprint 4 day 27 and 28
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,11 @@
           <t>ABB</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Abbott India Ltd</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -510,7 +514,11 @@
           <t>ADANIENSOL</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Adani Energy Solutions Ltd</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -546,7 +554,11 @@
           <t>ADANIENT</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Adani Enterprises Ltd</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -582,7 +594,11 @@
           <t>ADANIGREEN</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Adani Green Energy Ltd</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -618,7 +634,11 @@
           <t>ADANIPORTS</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Adani Ports &amp; Special Economic Zone Ltd</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -654,7 +674,11 @@
           <t>ADANIPOWER</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Adani Power Ltd</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -690,7 +714,11 @@
           <t>AMBUJACEM</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ambuja Cements Ltd</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -726,7 +754,12 @@
           <t>APOLLOHOSP</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals
+Chain of Indian private hospitals</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>Healthcare</t>
@@ -762,7 +795,12 @@
           <t>ASIANPAINT</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Asian Paints
+Indian Multi-National Paint and Coating Manufacturing Company</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -798,7 +836,11 @@
           <t>ATGL</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Adani Total Gas Ltd</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -832,7 +874,11 @@
           <t>AXISBANK</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Axis Bank Ltd</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -868,7 +914,11 @@
           <t>BAJAJ-AUTO</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bajaj Auto Ltd</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -904,7 +954,11 @@
           <t>BAJAJFINSV</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bajaj Finserv Ltd</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -940,7 +994,11 @@
           <t>BAJAJHLDNG</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bajaj Holdings &amp; Investment Ltd</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -976,7 +1034,11 @@
           <t>BAJFINANCE</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bajaj Finance Ltd</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1012,7 +1074,11 @@
           <t>BANKBARODA</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bank of Baroda</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1048,7 +1114,11 @@
           <t>BEL</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bharat Electronics Ltd</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -1084,7 +1154,11 @@
           <t>BHARTIARTL</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Ltd</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>Communication Services</t>
@@ -1120,7 +1194,11 @@
           <t>BHEL</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bharat Heavy Electricals Limited</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -1156,7 +1234,11 @@
           <t>BOSCHLTD</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bosch Ltd</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -1192,7 +1274,11 @@
           <t>BPCL</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bharat Petroleum Corporation Ltd</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -1228,7 +1314,11 @@
           <t>BRITANNIA</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Britannia Industries Ltd</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -1264,7 +1354,11 @@
           <t>CANBK</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Canara Bank</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1300,7 +1394,11 @@
           <t>CHOLAFIN</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1336,7 +1434,11 @@
           <t>CIPLA</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cipla Ltd</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>Healthcare</t>
@@ -1372,7 +1474,11 @@
           <t>COALINDIA</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Coal India Ltd</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -1408,7 +1514,11 @@
           <t>DABUR</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dabur India Ltd</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -1444,7 +1554,11 @@
           <t>DIVISLAB</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Divis Laboratories Ltd</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>Healthcare</t>
@@ -1480,7 +1594,11 @@
           <t>DLF</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DLF Ltd</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>Real Estate</t>
@@ -1516,7 +1634,11 @@
           <t>DMART</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Avenue Supermarts Ltd</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -1552,7 +1674,11 @@
           <t>DRREDDY</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Dr Reddys Laboratories Ltd</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>Healthcare</t>
@@ -1588,7 +1714,11 @@
           <t>EICHERMOT</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Eicher Motors Ltd</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -1624,7 +1754,11 @@
           <t>GAIL</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>GAIL (India) Ltd</t>
+        </is>
+      </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -1660,7 +1794,11 @@
           <t>GODREJCP</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Godrej Consumer Products Ltd</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -1696,7 +1834,11 @@
           <t>GRASIM</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Grasim Industries Ltd</t>
+        </is>
+      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -1732,7 +1874,11 @@
           <t>HAL</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Hindustan Aeronautics Ltd</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -1768,7 +1914,11 @@
           <t>HAVELLS</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Havells India Ltd</t>
+        </is>
+      </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -1804,7 +1954,11 @@
           <t>HCLTECH</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HCL Technologies Ltd</t>
+        </is>
+      </c>
       <c r="C39" t="inlineStr">
         <is>
           <t>Information Technology</t>
@@ -1840,7 +1994,11 @@
           <t>HDFCBANK</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HDFC Bank Ltd</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1876,7 +2034,11 @@
           <t>HDFCLIFE</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HDFC Life Insurance Company Ltd</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -1912,7 +2074,11 @@
           <t>HEROMOTOCO</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Hero MotoCorp Ltd</t>
+        </is>
+      </c>
       <c r="C42" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -1948,7 +2114,11 @@
           <t>HINDALCO</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Hindalco Industries Ltd</t>
+        </is>
+      </c>
       <c r="C43" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -1984,7 +2154,11 @@
           <t>HINDUNILVR</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Hindustan Unilever Ltd</t>
+        </is>
+      </c>
       <c r="C44" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -2020,7 +2194,11 @@
           <t>ICICIBANK</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ICICI Bank Ltd</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2056,7 +2234,11 @@
           <t>ICICIGI</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ICICI Lombard General Insurance Company Ltd</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2092,7 +2274,11 @@
           <t>ICICIPRULI</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ICICI Prudential Life Insurance Company Ltd</t>
+        </is>
+      </c>
       <c r="C47" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2128,7 +2314,11 @@
           <t>INDIGO</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Interglobe Aviation Ltd</t>
+        </is>
+      </c>
       <c r="C48" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -2164,7 +2354,11 @@
           <t>INDUSINDBK</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>IndusInd Bank Ltd</t>
+        </is>
+      </c>
       <c r="C49" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2200,7 +2394,11 @@
           <t>INFY</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Infosys Ltd</t>
+        </is>
+      </c>
       <c r="C50" t="inlineStr">
         <is>
           <t>Information Technology</t>
@@ -2236,7 +2434,11 @@
           <t>IOC</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Indian Oil Corporation</t>
+        </is>
+      </c>
       <c r="C51" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -2272,7 +2474,11 @@
           <t>IRCTC</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
+        </is>
+      </c>
       <c r="C52" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -2308,7 +2514,11 @@
           <t>IRFC</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Indian Railway Finance Corporation Ltd</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2344,7 +2554,11 @@
           <t>ITC</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ITC Ltd</t>
+        </is>
+      </c>
       <c r="C54" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -2380,7 +2594,11 @@
           <t>JINDALSTEL</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Jindal Steel &amp; Power Ltd</t>
+        </is>
+      </c>
       <c r="C55" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -2416,7 +2634,11 @@
           <t>JIOFIN</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Jio Financial Services Ltd</t>
+        </is>
+      </c>
       <c r="C56" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2452,7 +2674,11 @@
           <t>JSWENERGY</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>JSW Energy Ltd</t>
+        </is>
+      </c>
       <c r="C57" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -2488,7 +2714,11 @@
           <t>JSWSTEEL</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JSW Steel Ltd</t>
+        </is>
+      </c>
       <c r="C58" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -2524,7 +2754,11 @@
           <t>KOTAKBANK</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Kotak Mahindra Bank Ltd</t>
+        </is>
+      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2560,7 +2794,11 @@
           <t>LICI</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Life Insurance Corporation of India</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -2596,7 +2834,11 @@
           <t>LODHA</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Macrotech Developers Ltd</t>
+        </is>
+      </c>
       <c r="C61" t="inlineStr">
         <is>
           <t>Real Estate</t>
@@ -2632,7 +2874,11 @@
           <t>LT</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro Ltd</t>
+        </is>
+      </c>
       <c r="C62" t="inlineStr">
         <is>
           <t>Industrials</t>
@@ -2668,7 +2914,11 @@
           <t>LTIM</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>LTIMindtree Ltd</t>
+        </is>
+      </c>
       <c r="C63" t="inlineStr">
         <is>
           <t>Information Technology</t>
@@ -2704,7 +2954,11 @@
           <t>M&amp;M</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Mahindra &amp; Mahindra Ltd</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -2740,7 +2994,11 @@
           <t>MARUTI</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Ltd</t>
+        </is>
+      </c>
       <c r="C65" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -2776,7 +3034,11 @@
           <t>MOTHERSON</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Samvardhana Motherson International Ltd</t>
+        </is>
+      </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -2812,7 +3074,11 @@
           <t>NAUKRI</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Info Edge (India) Ltd</t>
+        </is>
+      </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>Communication Services</t>
@@ -2848,7 +3114,11 @@
           <t>NESTLEIND</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Nestle India Ltd</t>
+        </is>
+      </c>
       <c r="C68" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
@@ -2884,7 +3154,11 @@
           <t>NHPC</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NHPC Ltd</t>
+        </is>
+      </c>
       <c r="C69" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -2920,7 +3194,11 @@
           <t>NTPC</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>NTPC Ltd</t>
+        </is>
+      </c>
       <c r="C70" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -2956,7 +3234,11 @@
           <t>ONGC</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Oil &amp; Natural Gas Corpn Ltd</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -2992,7 +3274,11 @@
           <t>PFC</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Power Finance Corporation Ltd</t>
+        </is>
+      </c>
       <c r="C72" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -3028,7 +3314,11 @@
           <t>PIDILITIND</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Pidilite Industries Ltd</t>
+        </is>
+      </c>
       <c r="C73" t="inlineStr">
         <is>
           <t>Materials</t>
@@ -3064,7 +3354,11 @@
           <t>PNB</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Punjab National Bank</t>
+        </is>
+      </c>
       <c r="C74" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -3100,7 +3394,11 @@
           <t>POWERGRID</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Power Grid Corporation of India Ltd</t>
+        </is>
+      </c>
       <c r="C75" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -3136,7 +3434,11 @@
           <t>RECLTD</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>REC Ltd</t>
+        </is>
+      </c>
       <c r="C76" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -3172,7 +3474,11 @@
           <t>RELIANCE</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Reliance Industries Ltd</t>
+        </is>
+      </c>
       <c r="C77" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -3208,7 +3514,11 @@
           <t>SBILIFE</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SBI Life Insurance Company Ltd</t>
+        </is>
+      </c>
       <c r="C78" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -3241,140 +3551,144 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr"/>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>25.87</v>
-      </c>
-      <c r="E79" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="F79" t="n">
-        <v>26.58</v>
-      </c>
-      <c r="G79" t="n">
-        <v>0.06115348347250073</v>
-      </c>
-      <c r="H79" t="n">
-        <v>25.87</v>
-      </c>
-      <c r="I79" t="n">
-        <v>-53.48795397339086</v>
-      </c>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Discount</t>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr"/>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Shree Cement Ltd</t>
+        </is>
+      </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>68.53</v>
+        <v>25.87</v>
       </c>
       <c r="E80" t="n">
-        <v>7.91</v>
+        <v>1.21</v>
       </c>
       <c r="F80" t="n">
-        <v>28.82</v>
+        <v>26.58</v>
       </c>
       <c r="G80" t="n">
-        <v>-3.608906905151208</v>
+        <v>0.06115348347250073</v>
       </c>
       <c r="H80" t="n">
-        <v>68.53</v>
+        <v>25.87</v>
       </c>
       <c r="I80" t="n">
-        <v>104.1406017277331</v>
+        <v>-53.48795397339086</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Shriram Finance Ltd</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>33.32</v>
+        <v>68.53</v>
       </c>
       <c r="E81" t="n">
-        <v>9.25</v>
+        <v>7.91</v>
       </c>
       <c r="F81" t="n">
-        <v>30.88</v>
+        <v>28.82</v>
       </c>
       <c r="G81" t="n">
-        <v>0.09804152402695152</v>
+        <v>-3.608906905151208</v>
       </c>
       <c r="H81" t="n">
-        <v>33.32</v>
+        <v>68.53</v>
       </c>
       <c r="I81" t="n">
-        <v>-29.33941257554873</v>
+        <v>104.1406017277331</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Fair</t>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr"/>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Siemens Ltd</t>
+        </is>
+      </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>37.9</v>
+        <v>33.32</v>
       </c>
       <c r="E82" t="n">
-        <v>6.71</v>
+        <v>9.25</v>
       </c>
       <c r="F82" t="n">
-        <v>21.41</v>
+        <v>30.88</v>
       </c>
       <c r="G82" t="n">
-        <v>0.8489189373413096</v>
+        <v>0.09804152402695152</v>
       </c>
       <c r="H82" t="n">
-        <v>37.9</v>
+        <v>33.32</v>
       </c>
       <c r="I82" t="n">
-        <v>-19.46451338716533</v>
+        <v>-29.33941257554873</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -3385,32 +3699,36 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr"/>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
+        </is>
+      </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>54.79</v>
+        <v>37.9</v>
       </c>
       <c r="E83" t="n">
-        <v>7.14</v>
+        <v>6.71</v>
       </c>
       <c r="F83" t="n">
-        <v>24.84</v>
+        <v>21.41</v>
       </c>
       <c r="G83" t="n">
-        <v>0.007417056977403794</v>
+        <v>0.8489189373413096</v>
       </c>
       <c r="H83" t="n">
-        <v>54.79</v>
+        <v>37.9</v>
       </c>
       <c r="I83" t="n">
-        <v>7.536800785083408</v>
+        <v>-19.46451338716533</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -3421,140 +3739,156 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr"/>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Tata Consumer Products Ltd</t>
+        </is>
+      </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>67.06999999999999</v>
+        <v>54.79</v>
       </c>
       <c r="E84" t="n">
-        <v>0.93</v>
+        <v>7.14</v>
       </c>
       <c r="F84" t="n">
-        <v>15.35</v>
+        <v>24.84</v>
       </c>
       <c r="G84" t="n">
-        <v>3.000651602734764</v>
+        <v>0.007417056977403794</v>
       </c>
       <c r="H84" t="n">
-        <v>67.06999999999999</v>
+        <v>54.79</v>
       </c>
       <c r="I84" t="n">
-        <v>76.47677937113535</v>
+        <v>7.536800785083408</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr"/>
+          <t>TATAMOTORS</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>14.5</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="E85" t="n">
-        <v>3.48</v>
+        <v>0.93</v>
       </c>
       <c r="F85" t="n">
-        <v>12.02</v>
+        <v>15.35</v>
       </c>
       <c r="G85" t="n">
-        <v>0.2166615750083587</v>
+        <v>3.000651602734764</v>
       </c>
       <c r="H85" t="n">
-        <v>14.5</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="I85" t="n">
-        <v>-67.71679839697205</v>
+        <v>76.47677937113535</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Discount</t>
+          <t>Caution</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr"/>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Tata Power Company Ltd</t>
+        </is>
+      </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>48.97</v>
+        <v>14.5</v>
       </c>
       <c r="E86" t="n">
-        <v>9.23</v>
+        <v>3.48</v>
       </c>
       <c r="F86" t="n">
-        <v>38.87</v>
+        <v>12.02</v>
       </c>
       <c r="G86" t="n">
-        <v>1.638533052351645</v>
+        <v>0.2166615750083587</v>
       </c>
       <c r="H86" t="n">
-        <v>48.97</v>
+        <v>14.5</v>
       </c>
       <c r="I86" t="n">
-        <v>-11.95613088816972</v>
+        <v>-67.71679839697205</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Fair</t>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr"/>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Tata Steel Ltd</t>
+        </is>
+      </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>78.69</v>
+        <v>48.97</v>
       </c>
       <c r="E87" t="n">
-        <v>6.08</v>
+        <v>9.23</v>
       </c>
       <c r="F87" t="n">
-        <v>29.94</v>
+        <v>38.87</v>
       </c>
       <c r="G87" t="n">
-        <v>8.293144565835005</v>
+        <v>1.638533052351645</v>
       </c>
       <c r="H87" t="n">
-        <v>78.69</v>
+        <v>48.97</v>
       </c>
       <c r="I87" t="n">
-        <v>23.66808109382366</v>
+        <v>-11.95613088816972</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -3565,32 +3899,36 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TECHM</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Ltd</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>57.4</v>
+        <v>78.69</v>
       </c>
       <c r="E88" t="n">
-        <v>7.43</v>
+        <v>6.08</v>
       </c>
       <c r="F88" t="n">
-        <v>7.85</v>
+        <v>29.94</v>
       </c>
       <c r="G88" t="n">
-        <v>0.1674227036387368</v>
+        <v>8.293144565835005</v>
       </c>
       <c r="H88" t="n">
-        <v>57.4</v>
+        <v>78.69</v>
       </c>
       <c r="I88" t="n">
-        <v>-9.790979097909801</v>
+        <v>23.66808109382366</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -3601,142 +3939,198 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr"/>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Ltd</t>
+        </is>
+      </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>10.13</v>
+        <v>57.4</v>
       </c>
       <c r="E89" t="n">
-        <v>10.51</v>
+        <v>7.43</v>
       </c>
       <c r="F89" t="n">
-        <v>21</v>
+        <v>7.85</v>
       </c>
       <c r="G89" t="n">
-        <v>0.0839572651499547</v>
+        <v>0.1674227036387368</v>
       </c>
       <c r="H89" t="n">
-        <v>10.13</v>
+        <v>57.4</v>
       </c>
       <c r="I89" t="n">
-        <v>-73.3456124194185</v>
+        <v>-9.790979097909801</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Discount</t>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TORNTPHARM</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr"/>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Titan Company Ltd</t>
+        </is>
+      </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>46.4</v>
+        <v>10.13</v>
       </c>
       <c r="E90" t="n">
-        <v>6.43</v>
+        <v>10.51</v>
       </c>
       <c r="F90" t="n">
-        <v>27.93</v>
+        <v>21</v>
       </c>
       <c r="G90" t="n">
-        <v>0.1660811237632738</v>
+        <v>0.0839572651499547</v>
       </c>
       <c r="H90" t="n">
-        <v>46.4</v>
+        <v>10.13</v>
       </c>
       <c r="I90" t="n">
-        <v>-1.402464938376546</v>
+        <v>-73.3456124194185</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Fair</t>
+          <t>Discount</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TRENT</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr"/>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Torrent Pharmaceuticals Ltd</t>
+        </is>
+      </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>8.65</v>
+        <v>46.4</v>
       </c>
       <c r="E91" t="n">
-        <v>11.82</v>
+        <v>6.43</v>
       </c>
       <c r="F91" t="n">
-        <v>34.65</v>
+        <v>27.93</v>
       </c>
       <c r="G91" t="n">
-        <v>0.1472024429514394</v>
+        <v>0.1660811237632738</v>
       </c>
       <c r="H91" t="n">
-        <v>8.65</v>
+        <v>46.4</v>
       </c>
       <c r="I91" t="n">
-        <v>-77.23983686357059</v>
+        <v>-1.402464938376546</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Discount</t>
+          <t>Fair</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Trent Ltd</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="E92" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="F92" t="n">
+        <v>34.65</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0.1472024429514394</v>
+      </c>
+      <c r="H92" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="I92" t="n">
+        <v>-77.23983686357059</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>TVSMOTOR</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr">
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>TVS Motor Company Ltd</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D92" t="n">
+      <c r="D93" t="n">
         <v>46.1</v>
       </c>
-      <c r="E92" t="n">
+      <c r="E93" t="n">
         <v>5.62</v>
       </c>
-      <c r="F92" t="n">
+      <c r="F93" t="n">
         <v>7.1</v>
       </c>
-      <c r="G92" t="n">
+      <c r="G93" t="n">
         <v>-0.8454886074536311</v>
       </c>
-      <c r="H92" t="n">
+      <c r="H93" t="n">
         <v>46.1</v>
       </c>
-      <c r="I92" t="n">
+      <c r="I93" t="n">
         <v>21.29982896987237</v>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="J93" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>

</xml_diff>